<commit_message>
Atualizando configurações do gráfico e workspace, incluindo ajustes nas forças de ligação e escala. Removendo arquivos temporários obsoletos e melhorando a formatação das notas. Ajustes nos notebooks de normalização de despesas e receitas, com correções nas datas e melhorias na estrutura dos dados. Adicionando novos arquivos de saída e ajustando referências internas.
</commit_message>
<xml_diff>
--- a/02-Referencias/ATUA/Maio/ATUA_despesas_fechamento_05-2026.xlsx
+++ b/02-Referencias/ATUA/Maio/ATUA_despesas_fechamento_05-2026.xlsx
@@ -16,7 +16,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="4">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="166" formatCode="#.##0,00"/>
+    <numFmt numFmtId="167" formatCode="DD/MM/YYYY"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -49,9 +54,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -686,24 +693,22 @@
           <t>ALUGUEL05/2026-GSL</t>
         </is>
       </c>
-      <c r="T2" t="n">
+      <c r="T2" s="2" t="n">
         <v>1003.5</v>
       </c>
-      <c r="U2" t="n">
-        <v>1003.5</v>
-      </c>
-      <c r="V2" t="n">
-        <v>1003.5</v>
+      <c r="U2" s="2" t="n">
+        <v>-1003.5</v>
+      </c>
+      <c r="V2" s="2" t="n">
+        <v>-1003.5</v>
       </c>
       <c r="W2" t="inlineStr">
         <is>
           <t>ADMINISTRATIVO/COMERCIAL</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>04/05/2026</t>
-        </is>
+      <c r="X2" s="3" t="n">
+        <v>46146</v>
       </c>
       <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="inlineStr"/>
@@ -826,24 +831,22 @@
           <t>231</t>
         </is>
       </c>
-      <c r="T3" t="n">
+      <c r="T3" s="2" t="n">
         <v>1545</v>
       </c>
-      <c r="U3" t="n">
-        <v>1545</v>
-      </c>
-      <c r="V3" t="n">
-        <v>1545</v>
+      <c r="U3" s="2" t="n">
+        <v>-1545</v>
+      </c>
+      <c r="V3" s="2" t="n">
+        <v>-1545</v>
       </c>
       <c r="W3" t="inlineStr">
         <is>
           <t>ADMINISTRATIVO/COMERCIAL</t>
         </is>
       </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>04/05/2026</t>
-        </is>
+      <c r="X3" s="3" t="n">
+        <v>46146</v>
       </c>
       <c r="Y3" t="inlineStr"/>
       <c r="Z3" t="inlineStr"/>
@@ -898,22 +901,22 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.4</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>BARUERI</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.4 BARUERI</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.4.2</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -923,12 +926,12 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.4.2 ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.4.2</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -938,7 +941,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.4.2 ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -958,7 +961,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>GSL PRUDENTE</t>
+          <t>GSL BARUERI</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -966,24 +969,22 @@
           <t>PRO-LAB 042026</t>
         </is>
       </c>
-      <c r="T4" t="n">
+      <c r="T4" s="2" t="n">
         <v>1442.69</v>
       </c>
-      <c r="U4" t="n">
-        <v>1442.69</v>
-      </c>
-      <c r="V4" t="n">
-        <v>1442.69</v>
+      <c r="U4" s="2" t="n">
+        <v>-1442.69</v>
+      </c>
+      <c r="V4" s="2" t="n">
+        <v>-1442.69</v>
       </c>
       <c r="W4" t="inlineStr">
         <is>
           <t>ADMINISTRATIVO/COMERCIAL</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t>06/05/2026</t>
-        </is>
+      <c r="X4" s="3" t="n">
+        <v>46148</v>
       </c>
       <c r="Y4" t="inlineStr"/>
       <c r="Z4" t="inlineStr"/>
@@ -1053,32 +1054,32 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>1.4.1.1</t>
+          <t>1.4.1.2</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>TRANSPORTE</t>
+          <t>ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>1.4.1.1 TRANSPORTE</t>
+          <t>1.4.1.2 ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>1.4.1.1</t>
+          <t>1.4.1.2</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>TRANSPORTE</t>
+          <t>ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>1.4.1.1 TRANSPORTE</t>
+          <t>1.4.1.2 ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -1106,24 +1107,22 @@
           <t>30874</t>
         </is>
       </c>
-      <c r="T5" t="n">
+      <c r="T5" s="2" t="n">
         <v>199</v>
       </c>
-      <c r="U5" t="n">
-        <v>199</v>
-      </c>
-      <c r="V5" t="n">
-        <v>199</v>
+      <c r="U5" s="2" t="n">
+        <v>-199</v>
+      </c>
+      <c r="V5" s="2" t="n">
+        <v>-199</v>
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>TRANSPORTE</t>
-        </is>
-      </c>
-      <c r="X5" t="inlineStr">
-        <is>
-          <t>06/05/2026</t>
-        </is>
+          <t>ADMINISTRATIVO/COMERCIAL</t>
+        </is>
+      </c>
+      <c r="X5" s="3" t="n">
+        <v>46148</v>
       </c>
       <c r="Y5" t="inlineStr"/>
       <c r="Z5" t="inlineStr"/>
@@ -1246,24 +1245,22 @@
           <t>666</t>
         </is>
       </c>
-      <c r="T6" t="n">
+      <c r="T6" s="2" t="n">
         <v>1671.35</v>
       </c>
-      <c r="U6" t="n">
-        <v>1671.35</v>
-      </c>
-      <c r="V6" t="n">
-        <v>1671.35</v>
+      <c r="U6" s="2" t="n">
+        <v>-1671.35</v>
+      </c>
+      <c r="V6" s="2" t="n">
+        <v>-1671.35</v>
       </c>
       <c r="W6" t="inlineStr">
         <is>
           <t>ADMINISTRATIVO/COMERCIAL</t>
         </is>
       </c>
-      <c r="X6" t="inlineStr">
-        <is>
-          <t>08/05/2026</t>
-        </is>
+      <c r="X6" s="3" t="n">
+        <v>46150</v>
       </c>
       <c r="Y6" t="inlineStr"/>
       <c r="Z6" t="inlineStr"/>
@@ -1386,24 +1383,22 @@
           <t>ICMS042026GSL02</t>
         </is>
       </c>
-      <c r="T7" t="n">
+      <c r="T7" s="2" t="n">
         <v>81994.42999999999</v>
       </c>
-      <c r="U7" t="n">
-        <v>81994.42999999999</v>
-      </c>
-      <c r="V7" t="n">
-        <v>81994.42999999999</v>
+      <c r="U7" s="2" t="n">
+        <v>-81994.42999999999</v>
+      </c>
+      <c r="V7" s="2" t="n">
+        <v>-81994.42999999999</v>
       </c>
       <c r="W7" t="inlineStr">
         <is>
           <t>ADMINISTRATIVO/COMERCIAL</t>
         </is>
       </c>
-      <c r="X7" t="inlineStr">
-        <is>
-          <t>08/05/2026</t>
-        </is>
+      <c r="X7" s="3" t="n">
+        <v>46150</v>
       </c>
       <c r="Y7" t="inlineStr"/>
       <c r="Z7" t="inlineStr"/>
@@ -1526,24 +1521,22 @@
           <t>ICMS042026GSL03</t>
         </is>
       </c>
-      <c r="T8" t="n">
+      <c r="T8" s="2" t="n">
         <v>13099.5</v>
       </c>
-      <c r="U8" t="n">
-        <v>13099.5</v>
-      </c>
-      <c r="V8" t="n">
-        <v>13099.5</v>
+      <c r="U8" s="2" t="n">
+        <v>-13099.5</v>
+      </c>
+      <c r="V8" s="2" t="n">
+        <v>-13099.5</v>
       </c>
       <c r="W8" t="inlineStr">
         <is>
           <t>ADMINISTRATIVO/COMERCIAL</t>
         </is>
       </c>
-      <c r="X8" t="inlineStr">
-        <is>
-          <t>08/05/2026</t>
-        </is>
+      <c r="X8" s="3" t="n">
+        <v>46150</v>
       </c>
       <c r="Y8" t="inlineStr"/>
       <c r="Z8" t="inlineStr"/>
@@ -1666,24 +1659,22 @@
           <t>ICMS042026GSL01</t>
         </is>
       </c>
-      <c r="T9" t="n">
+      <c r="T9" s="2" t="n">
         <v>163583.3</v>
       </c>
-      <c r="U9" t="n">
-        <v>163583.3</v>
-      </c>
-      <c r="V9" t="n">
-        <v>163583.3</v>
+      <c r="U9" s="2" t="n">
+        <v>-163583.3</v>
+      </c>
+      <c r="V9" s="2" t="n">
+        <v>-163583.3</v>
       </c>
       <c r="W9" t="inlineStr">
         <is>
           <t>ADMINISTRATIVO/COMERCIAL</t>
         </is>
       </c>
-      <c r="X9" t="inlineStr">
-        <is>
-          <t>08/05/2026</t>
-        </is>
+      <c r="X9" s="3" t="n">
+        <v>46150</v>
       </c>
       <c r="Y9" t="inlineStr"/>
       <c r="Z9" t="inlineStr"/>
@@ -1753,32 +1744,32 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -1806,24 +1797,22 @@
           <t>32940</t>
         </is>
       </c>
-      <c r="T10" t="n">
+      <c r="T10" s="2" t="n">
         <v>113.97</v>
       </c>
-      <c r="U10" t="n">
-        <v>113.97</v>
-      </c>
-      <c r="V10" t="n">
-        <v>113.97</v>
+      <c r="U10" s="2" t="n">
+        <v>-113.97</v>
+      </c>
+      <c r="V10" s="2" t="n">
+        <v>-113.97</v>
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO/COMERCIAL</t>
-        </is>
-      </c>
-      <c r="X10" t="inlineStr">
-        <is>
-          <t>11/05/2026</t>
-        </is>
+          <t>FROTA TERCEIRO PRUDENTE</t>
+        </is>
+      </c>
+      <c r="X10" s="3" t="n">
+        <v>46153</v>
       </c>
       <c r="Y10" t="inlineStr"/>
       <c r="Z10" t="inlineStr"/>
@@ -1893,32 +1882,32 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -1946,24 +1935,22 @@
           <t>32534</t>
         </is>
       </c>
-      <c r="T11" t="n">
+      <c r="T11" s="2" t="n">
         <v>625.48</v>
       </c>
-      <c r="U11" t="n">
-        <v>625.48</v>
-      </c>
-      <c r="V11" t="n">
-        <v>625.48</v>
+      <c r="U11" s="2" t="n">
+        <v>-625.48</v>
+      </c>
+      <c r="V11" s="2" t="n">
+        <v>-625.48</v>
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO/COMERCIAL</t>
-        </is>
-      </c>
-      <c r="X11" t="inlineStr">
-        <is>
-          <t>11/05/2026</t>
-        </is>
+          <t>FROTA TERCEIRO PRUDENTE</t>
+        </is>
+      </c>
+      <c r="X11" s="3" t="n">
+        <v>46153</v>
       </c>
       <c r="Y11" t="inlineStr"/>
       <c r="Z11" t="inlineStr"/>
@@ -2033,32 +2020,32 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
@@ -2086,24 +2073,22 @@
           <t>34293</t>
         </is>
       </c>
-      <c r="T12" t="n">
+      <c r="T12" s="2" t="n">
         <v>444.26</v>
       </c>
-      <c r="U12" t="n">
-        <v>444.26</v>
-      </c>
-      <c r="V12" t="n">
-        <v>444.26</v>
+      <c r="U12" s="2" t="n">
+        <v>-444.26</v>
+      </c>
+      <c r="V12" s="2" t="n">
+        <v>-444.26</v>
       </c>
       <c r="W12" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO/COMERCIAL</t>
-        </is>
-      </c>
-      <c r="X12" t="inlineStr">
-        <is>
-          <t>11/05/2026</t>
-        </is>
+          <t>FROTA TERCEIRO PRUDENTE</t>
+        </is>
+      </c>
+      <c r="X12" s="3" t="n">
+        <v>46153</v>
       </c>
       <c r="Y12" t="inlineStr"/>
       <c r="Z12" t="inlineStr"/>
@@ -2173,32 +2158,32 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -2226,24 +2211,22 @@
           <t>35116</t>
         </is>
       </c>
-      <c r="T13" t="n">
+      <c r="T13" s="2" t="n">
         <v>714.6</v>
       </c>
-      <c r="U13" t="n">
-        <v>714.6</v>
-      </c>
-      <c r="V13" t="n">
-        <v>714.6</v>
+      <c r="U13" s="2" t="n">
+        <v>-714.6</v>
+      </c>
+      <c r="V13" s="2" t="n">
+        <v>-714.6</v>
       </c>
       <c r="W13" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO/COMERCIAL</t>
-        </is>
-      </c>
-      <c r="X13" t="inlineStr">
-        <is>
-          <t>11/05/2026</t>
-        </is>
+          <t>FROTA TERCEIRO PRUDENTE</t>
+        </is>
+      </c>
+      <c r="X13" s="3" t="n">
+        <v>46153</v>
       </c>
       <c r="Y13" t="inlineStr"/>
       <c r="Z13" t="inlineStr"/>
@@ -2298,47 +2281,47 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>1.4.3</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>MARINGA</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>1.4.3 MARINGA</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>1.4.3.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>1.4.3.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>1.4.3.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>1.4.3.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
@@ -2358,7 +2341,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>GSL MARINGA</t>
+          <t>GSL PRUDENTE</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -2366,24 +2349,22 @@
           <t>35696</t>
         </is>
       </c>
-      <c r="T14" t="n">
+      <c r="T14" s="2" t="n">
         <v>175.8</v>
       </c>
-      <c r="U14" t="n">
-        <v>175.8</v>
-      </c>
-      <c r="V14" t="n">
-        <v>175.8</v>
+      <c r="U14" s="2" t="n">
+        <v>-175.8</v>
+      </c>
+      <c r="V14" s="2" t="n">
+        <v>-175.8</v>
       </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO/COMERCIAL</t>
-        </is>
-      </c>
-      <c r="X14" t="inlineStr">
-        <is>
-          <t>11/05/2026</t>
-        </is>
+          <t>FROTA TERCEIRO PRUDENTE</t>
+        </is>
+      </c>
+      <c r="X14" s="3" t="n">
+        <v>46153</v>
       </c>
       <c r="Y14" t="inlineStr"/>
       <c r="Z14" t="inlineStr"/>
@@ -2453,32 +2434,32 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
@@ -2506,24 +2487,22 @@
           <t>36293</t>
         </is>
       </c>
-      <c r="T15" t="n">
+      <c r="T15" s="2" t="n">
         <v>490.94</v>
       </c>
-      <c r="U15" t="n">
-        <v>490.94</v>
-      </c>
-      <c r="V15" t="n">
-        <v>490.94</v>
+      <c r="U15" s="2" t="n">
+        <v>-490.94</v>
+      </c>
+      <c r="V15" s="2" t="n">
+        <v>-490.94</v>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO/COMERCIAL</t>
-        </is>
-      </c>
-      <c r="X15" t="inlineStr">
-        <is>
-          <t>11/05/2026</t>
-        </is>
+          <t>FROTA TERCEIRO PRUDENTE</t>
+        </is>
+      </c>
+      <c r="X15" s="3" t="n">
+        <v>46153</v>
       </c>
       <c r="Y15" t="inlineStr"/>
       <c r="Z15" t="inlineStr"/>
@@ -2593,32 +2572,32 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -2646,24 +2625,22 @@
           <t>36898</t>
         </is>
       </c>
-      <c r="T16" t="n">
+      <c r="T16" s="2" t="n">
         <v>407.26</v>
       </c>
-      <c r="U16" t="n">
-        <v>407.26</v>
-      </c>
-      <c r="V16" t="n">
-        <v>407.26</v>
+      <c r="U16" s="2" t="n">
+        <v>-407.26</v>
+      </c>
+      <c r="V16" s="2" t="n">
+        <v>-407.26</v>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO/COMERCIAL</t>
-        </is>
-      </c>
-      <c r="X16" t="inlineStr">
-        <is>
-          <t>11/05/2026</t>
-        </is>
+          <t>FROTA TERCEIRO PRUDENTE</t>
+        </is>
+      </c>
+      <c r="X16" s="3" t="n">
+        <v>46153</v>
       </c>
       <c r="Y16" t="inlineStr"/>
       <c r="Z16" t="inlineStr"/>
@@ -2786,24 +2763,22 @@
           <t>939</t>
         </is>
       </c>
-      <c r="T17" t="n">
+      <c r="T17" s="2" t="n">
         <v>1018.78</v>
       </c>
-      <c r="U17" t="n">
-        <v>1018.78</v>
-      </c>
-      <c r="V17" t="n">
-        <v>1018.78</v>
+      <c r="U17" s="2" t="n">
+        <v>-1018.78</v>
+      </c>
+      <c r="V17" s="2" t="n">
+        <v>-1018.78</v>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>TRANSPORTE</t>
-        </is>
-      </c>
-      <c r="X17" t="inlineStr">
-        <is>
-          <t>11/05/2026</t>
-        </is>
+          <t>FROTA TERCEIRO PRUDENTE</t>
+        </is>
+      </c>
+      <c r="X17" s="3" t="n">
+        <v>46153</v>
       </c>
       <c r="Y17" t="inlineStr"/>
       <c r="Z17" t="inlineStr"/>
@@ -2926,24 +2901,22 @@
           <t>259</t>
         </is>
       </c>
-      <c r="T18" t="n">
+      <c r="T18" s="2" t="n">
         <v>1848.77</v>
       </c>
-      <c r="U18" t="n">
-        <v>1848.77</v>
-      </c>
-      <c r="V18" t="n">
-        <v>1848.77</v>
+      <c r="U18" s="2" t="n">
+        <v>-1848.77</v>
+      </c>
+      <c r="V18" s="2" t="n">
+        <v>-1848.77</v>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>TRANSPORTE</t>
-        </is>
-      </c>
-      <c r="X18" t="inlineStr">
-        <is>
-          <t>11/05/2026</t>
-        </is>
+          <t>FROTA TERCEIRO PRUDENTE</t>
+        </is>
+      </c>
+      <c r="X18" s="3" t="n">
+        <v>46153</v>
       </c>
       <c r="Y18" t="inlineStr"/>
       <c r="Z18" t="inlineStr"/>
@@ -3066,24 +3039,22 @@
           <t>983</t>
         </is>
       </c>
-      <c r="T19" t="n">
+      <c r="T19" s="2" t="n">
         <v>391.26</v>
       </c>
-      <c r="U19" t="n">
-        <v>391.26</v>
-      </c>
-      <c r="V19" t="n">
-        <v>391.26</v>
+      <c r="U19" s="2" t="n">
+        <v>-391.26</v>
+      </c>
+      <c r="V19" s="2" t="n">
+        <v>-391.26</v>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>TRANSPORTE</t>
-        </is>
-      </c>
-      <c r="X19" t="inlineStr">
-        <is>
-          <t>11/05/2026</t>
-        </is>
+          <t>FROTA TERCEIRO PRUDENTE</t>
+        </is>
+      </c>
+      <c r="X19" s="3" t="n">
+        <v>46153</v>
       </c>
       <c r="Y19" t="inlineStr"/>
       <c r="Z19" t="inlineStr"/>
@@ -3153,32 +3124,32 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
@@ -3206,24 +3177,22 @@
           <t>TRPED90426</t>
         </is>
       </c>
-      <c r="T20" t="n">
+      <c r="T20" s="2" t="n">
         <v>44.96</v>
       </c>
-      <c r="U20" t="n">
-        <v>44.96</v>
-      </c>
-      <c r="V20" t="n">
-        <v>44.96</v>
+      <c r="U20" s="2" t="n">
+        <v>-44.96</v>
+      </c>
+      <c r="V20" s="2" t="n">
+        <v>-44.96</v>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO/COMERCIAL</t>
-        </is>
-      </c>
-      <c r="X20" t="inlineStr">
-        <is>
-          <t>12/05/2026</t>
-        </is>
+          <t>FROTA TERCEIRO PRUDENTE</t>
+        </is>
+      </c>
+      <c r="X20" s="3" t="n">
+        <v>46154</v>
       </c>
       <c r="Y20" t="inlineStr"/>
       <c r="Z20" t="inlineStr"/>
@@ -3293,32 +3262,32 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
@@ -3346,24 +3315,22 @@
           <t>TRPED100426</t>
         </is>
       </c>
-      <c r="T21" t="n">
+      <c r="T21" s="2" t="n">
         <v>39.28</v>
       </c>
-      <c r="U21" t="n">
-        <v>39.28</v>
-      </c>
-      <c r="V21" t="n">
-        <v>39.28</v>
+      <c r="U21" s="2" t="n">
+        <v>-39.28</v>
+      </c>
+      <c r="V21" s="2" t="n">
+        <v>-39.28</v>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO/COMERCIAL</t>
-        </is>
-      </c>
-      <c r="X21" t="inlineStr">
-        <is>
-          <t>12/05/2026</t>
-        </is>
+          <t>FROTA TERCEIRO PRUDENTE</t>
+        </is>
+      </c>
+      <c r="X21" s="3" t="n">
+        <v>46154</v>
       </c>
       <c r="Y21" t="inlineStr"/>
       <c r="Z21" t="inlineStr"/>
@@ -3433,32 +3400,32 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
@@ -3486,24 +3453,22 @@
           <t>TRPED110426</t>
         </is>
       </c>
-      <c r="T22" t="n">
+      <c r="T22" s="2" t="n">
         <v>23.44</v>
       </c>
-      <c r="U22" t="n">
-        <v>23.44</v>
-      </c>
-      <c r="V22" t="n">
-        <v>23.44</v>
+      <c r="U22" s="2" t="n">
+        <v>-23.44</v>
+      </c>
+      <c r="V22" s="2" t="n">
+        <v>-23.44</v>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO/COMERCIAL</t>
-        </is>
-      </c>
-      <c r="X22" t="inlineStr">
-        <is>
-          <t>12/05/2026</t>
-        </is>
+          <t>FROTA TERCEIRO PRUDENTE</t>
+        </is>
+      </c>
+      <c r="X22" s="3" t="n">
+        <v>46154</v>
       </c>
       <c r="Y22" t="inlineStr"/>
       <c r="Z22" t="inlineStr"/>
@@ -3573,32 +3538,32 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
@@ -3626,24 +3591,22 @@
           <t>TRPED120426</t>
         </is>
       </c>
-      <c r="T23" t="n">
+      <c r="T23" s="2" t="n">
         <v>3.13</v>
       </c>
-      <c r="U23" t="n">
-        <v>3.13</v>
-      </c>
-      <c r="V23" t="n">
-        <v>3.13</v>
+      <c r="U23" s="2" t="n">
+        <v>-3.13</v>
+      </c>
+      <c r="V23" s="2" t="n">
+        <v>-3.13</v>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO/COMERCIAL</t>
-        </is>
-      </c>
-      <c r="X23" t="inlineStr">
-        <is>
-          <t>12/05/2026</t>
-        </is>
+          <t>FROTA TERCEIRO PRUDENTE</t>
+        </is>
+      </c>
+      <c r="X23" s="3" t="n">
+        <v>46154</v>
       </c>
       <c r="Y23" t="inlineStr"/>
       <c r="Z23" t="inlineStr"/>
@@ -3713,32 +3676,32 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
@@ -3766,24 +3729,22 @@
           <t>TRPED130426</t>
         </is>
       </c>
-      <c r="T24" t="n">
+      <c r="T24" s="2" t="n">
         <v>35.25</v>
       </c>
-      <c r="U24" t="n">
-        <v>35.25</v>
-      </c>
-      <c r="V24" t="n">
-        <v>35.25</v>
+      <c r="U24" s="2" t="n">
+        <v>-35.25</v>
+      </c>
+      <c r="V24" s="2" t="n">
+        <v>-35.25</v>
       </c>
       <c r="W24" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO/COMERCIAL</t>
-        </is>
-      </c>
-      <c r="X24" t="inlineStr">
-        <is>
-          <t>12/05/2026</t>
-        </is>
+          <t>FROTA TERCEIRO PRUDENTE</t>
+        </is>
+      </c>
+      <c r="X24" s="3" t="n">
+        <v>46154</v>
       </c>
       <c r="Y24" t="inlineStr"/>
       <c r="Z24" t="inlineStr"/>
@@ -3853,32 +3814,32 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
@@ -3906,24 +3867,22 @@
           <t>TRPED140426</t>
         </is>
       </c>
-      <c r="T25" t="n">
+      <c r="T25" s="2" t="n">
         <v>68.08</v>
       </c>
-      <c r="U25" t="n">
-        <v>68.08</v>
-      </c>
-      <c r="V25" t="n">
-        <v>68.08</v>
+      <c r="U25" s="2" t="n">
+        <v>-68.08</v>
+      </c>
+      <c r="V25" s="2" t="n">
+        <v>-68.08</v>
       </c>
       <c r="W25" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO/COMERCIAL</t>
-        </is>
-      </c>
-      <c r="X25" t="inlineStr">
-        <is>
-          <t>12/05/2026</t>
-        </is>
+          <t>FROTA TERCEIRO PRUDENTE</t>
+        </is>
+      </c>
+      <c r="X25" s="3" t="n">
+        <v>46154</v>
       </c>
       <c r="Y25" t="inlineStr"/>
       <c r="Z25" t="inlineStr"/>
@@ -3993,32 +3952,32 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
@@ -4046,24 +4005,22 @@
           <t>TRPED150526</t>
         </is>
       </c>
-      <c r="T26" t="n">
+      <c r="T26" s="2" t="n">
         <v>33.37</v>
       </c>
-      <c r="U26" t="n">
-        <v>33.37</v>
-      </c>
-      <c r="V26" t="n">
-        <v>33.37</v>
+      <c r="U26" s="2" t="n">
+        <v>-33.37</v>
+      </c>
+      <c r="V26" s="2" t="n">
+        <v>-33.37</v>
       </c>
       <c r="W26" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO/COMERCIAL</t>
-        </is>
-      </c>
-      <c r="X26" t="inlineStr">
-        <is>
-          <t>12/05/2026</t>
-        </is>
+          <t>FROTA TERCEIRO PRUDENTE</t>
+        </is>
+      </c>
+      <c r="X26" s="3" t="n">
+        <v>46154</v>
       </c>
       <c r="Y26" t="inlineStr"/>
       <c r="Z26" t="inlineStr"/>
@@ -4133,32 +4090,32 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
@@ -4186,24 +4143,22 @@
           <t>TRPED160426</t>
         </is>
       </c>
-      <c r="T27" t="n">
+      <c r="T27" s="2" t="n">
         <v>45.04</v>
       </c>
-      <c r="U27" t="n">
-        <v>45.04</v>
-      </c>
-      <c r="V27" t="n">
-        <v>45.04</v>
+      <c r="U27" s="2" t="n">
+        <v>-45.04</v>
+      </c>
+      <c r="V27" s="2" t="n">
+        <v>-45.04</v>
       </c>
       <c r="W27" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO/COMERCIAL</t>
-        </is>
-      </c>
-      <c r="X27" t="inlineStr">
-        <is>
-          <t>12/05/2026</t>
-        </is>
+          <t>FROTA TERCEIRO PRUDENTE</t>
+        </is>
+      </c>
+      <c r="X27" s="3" t="n">
+        <v>46154</v>
       </c>
       <c r="Y27" t="inlineStr"/>
       <c r="Z27" t="inlineStr"/>
@@ -4326,24 +4281,22 @@
           <t>468385</t>
         </is>
       </c>
-      <c r="T28" t="n">
+      <c r="T28" s="2" t="n">
         <v>6458.58</v>
       </c>
-      <c r="U28" t="n">
-        <v>6458.58</v>
-      </c>
-      <c r="V28" t="n">
-        <v>6458.58</v>
+      <c r="U28" s="2" t="n">
+        <v>-6458.58</v>
+      </c>
+      <c r="V28" s="2" t="n">
+        <v>-6458.58</v>
       </c>
       <c r="W28" t="inlineStr">
         <is>
           <t>ADMINISTRATIVO/COMERCIAL</t>
         </is>
       </c>
-      <c r="X28" t="inlineStr">
-        <is>
-          <t>13/05/2026</t>
-        </is>
+      <c r="X28" s="3" t="n">
+        <v>46155</v>
       </c>
       <c r="Y28" t="inlineStr"/>
       <c r="Z28" t="inlineStr"/>
@@ -4413,32 +4366,32 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
@@ -4466,24 +4419,22 @@
           <t>TRPED170426</t>
         </is>
       </c>
-      <c r="T29" t="n">
+      <c r="T29" s="2" t="n">
         <v>69.11</v>
       </c>
-      <c r="U29" t="n">
-        <v>69.11</v>
-      </c>
-      <c r="V29" t="n">
-        <v>69.11</v>
+      <c r="U29" s="2" t="n">
+        <v>-69.11</v>
+      </c>
+      <c r="V29" s="2" t="n">
+        <v>-69.11</v>
       </c>
       <c r="W29" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO/COMERCIAL</t>
-        </is>
-      </c>
-      <c r="X29" t="inlineStr">
-        <is>
-          <t>13/05/2026</t>
-        </is>
+          <t>FROTA TERCEIRO PRUDENTE</t>
+        </is>
+      </c>
+      <c r="X29" s="3" t="n">
+        <v>46155</v>
       </c>
       <c r="Y29" t="inlineStr"/>
       <c r="Z29" t="inlineStr"/>
@@ -4553,32 +4504,32 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
@@ -4606,24 +4557,22 @@
           <t>TRPED200426</t>
         </is>
       </c>
-      <c r="T30" t="n">
+      <c r="T30" s="2" t="n">
         <v>28.94</v>
       </c>
-      <c r="U30" t="n">
-        <v>28.94</v>
-      </c>
-      <c r="V30" t="n">
-        <v>28.94</v>
+      <c r="U30" s="2" t="n">
+        <v>-28.94</v>
+      </c>
+      <c r="V30" s="2" t="n">
+        <v>-28.94</v>
       </c>
       <c r="W30" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO/COMERCIAL</t>
-        </is>
-      </c>
-      <c r="X30" t="inlineStr">
-        <is>
-          <t>13/05/2026</t>
-        </is>
+          <t>FROTA TERCEIRO PRUDENTE</t>
+        </is>
+      </c>
+      <c r="X30" s="3" t="n">
+        <v>46155</v>
       </c>
       <c r="Y30" t="inlineStr"/>
       <c r="Z30" t="inlineStr"/>
@@ -4693,32 +4642,32 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
@@ -4746,24 +4695,22 @@
           <t>TRPED210426</t>
         </is>
       </c>
-      <c r="T31" t="n">
+      <c r="T31" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="U31" t="n">
-        <v>3</v>
-      </c>
-      <c r="V31" t="n">
-        <v>3</v>
+      <c r="U31" s="2" t="n">
+        <v>-3</v>
+      </c>
+      <c r="V31" s="2" t="n">
+        <v>-3</v>
       </c>
       <c r="W31" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO/COMERCIAL</t>
-        </is>
-      </c>
-      <c r="X31" t="inlineStr">
-        <is>
-          <t>13/05/2026</t>
-        </is>
+          <t>FROTA TERCEIRO PRUDENTE</t>
+        </is>
+      </c>
+      <c r="X31" s="3" t="n">
+        <v>46155</v>
       </c>
       <c r="Y31" t="inlineStr"/>
       <c r="Z31" t="inlineStr"/>
@@ -4833,32 +4780,32 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
@@ -4886,24 +4833,22 @@
           <t>TRPED220426</t>
         </is>
       </c>
-      <c r="T32" t="n">
+      <c r="T32" s="2" t="n">
         <v>34.05</v>
       </c>
-      <c r="U32" t="n">
-        <v>34.05</v>
-      </c>
-      <c r="V32" t="n">
-        <v>34.05</v>
+      <c r="U32" s="2" t="n">
+        <v>-34.05</v>
+      </c>
+      <c r="V32" s="2" t="n">
+        <v>-34.05</v>
       </c>
       <c r="W32" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO/COMERCIAL</t>
-        </is>
-      </c>
-      <c r="X32" t="inlineStr">
-        <is>
-          <t>13/05/2026</t>
-        </is>
+          <t>FROTA TERCEIRO PRUDENTE</t>
+        </is>
+      </c>
+      <c r="X32" s="3" t="n">
+        <v>46155</v>
       </c>
       <c r="Y32" t="inlineStr"/>
       <c r="Z32" t="inlineStr"/>
@@ -4973,32 +4918,32 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
@@ -5026,24 +4971,22 @@
           <t>TRPED230426</t>
         </is>
       </c>
-      <c r="T33" t="n">
+      <c r="T33" s="2" t="n">
         <v>58.08</v>
       </c>
-      <c r="U33" t="n">
-        <v>58.08</v>
-      </c>
-      <c r="V33" t="n">
-        <v>58.08</v>
+      <c r="U33" s="2" t="n">
+        <v>-58.08</v>
+      </c>
+      <c r="V33" s="2" t="n">
+        <v>-58.08</v>
       </c>
       <c r="W33" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO/COMERCIAL</t>
-        </is>
-      </c>
-      <c r="X33" t="inlineStr">
-        <is>
-          <t>13/05/2026</t>
-        </is>
+          <t>FROTA TERCEIRO PRUDENTE</t>
+        </is>
+      </c>
+      <c r="X33" s="3" t="n">
+        <v>46155</v>
       </c>
       <c r="Y33" t="inlineStr"/>
       <c r="Z33" t="inlineStr"/>
@@ -5113,32 +5056,32 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
@@ -5166,24 +5109,22 @@
           <t>TRPED240426</t>
         </is>
       </c>
-      <c r="T34" t="n">
+      <c r="T34" s="2" t="n">
         <v>46.11</v>
       </c>
-      <c r="U34" t="n">
-        <v>46.11</v>
-      </c>
-      <c r="V34" t="n">
-        <v>46.11</v>
+      <c r="U34" s="2" t="n">
+        <v>-46.11</v>
+      </c>
+      <c r="V34" s="2" t="n">
+        <v>-46.11</v>
       </c>
       <c r="W34" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO/COMERCIAL</t>
-        </is>
-      </c>
-      <c r="X34" t="inlineStr">
-        <is>
-          <t>15/05/2026</t>
-        </is>
+          <t>FROTA TERCEIRO PRUDENTE</t>
+        </is>
+      </c>
+      <c r="X34" s="3" t="n">
+        <v>46157</v>
       </c>
       <c r="Y34" t="inlineStr"/>
       <c r="Z34" t="inlineStr"/>
@@ -5253,32 +5194,32 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
@@ -5306,24 +5247,22 @@
           <t>TRPED270426</t>
         </is>
       </c>
-      <c r="T35" t="n">
+      <c r="T35" s="2" t="n">
         <v>51.78</v>
       </c>
-      <c r="U35" t="n">
-        <v>51.78</v>
-      </c>
-      <c r="V35" t="n">
-        <v>51.78</v>
+      <c r="U35" s="2" t="n">
+        <v>-51.78</v>
+      </c>
+      <c r="V35" s="2" t="n">
+        <v>-51.78</v>
       </c>
       <c r="W35" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO/COMERCIAL</t>
-        </is>
-      </c>
-      <c r="X35" t="inlineStr">
-        <is>
-          <t>15/05/2026</t>
-        </is>
+          <t>FROTA TERCEIRO PRUDENTE</t>
+        </is>
+      </c>
+      <c r="X35" s="3" t="n">
+        <v>46157</v>
       </c>
       <c r="Y35" t="inlineStr"/>
       <c r="Z35" t="inlineStr"/>
@@ -5393,32 +5332,32 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
@@ -5446,24 +5385,22 @@
           <t>TRPED280426</t>
         </is>
       </c>
-      <c r="T36" t="n">
+      <c r="T36" s="2" t="n">
         <v>60.06</v>
       </c>
-      <c r="U36" t="n">
-        <v>60.06</v>
-      </c>
-      <c r="V36" t="n">
-        <v>60.06</v>
+      <c r="U36" s="2" t="n">
+        <v>-60.06</v>
+      </c>
+      <c r="V36" s="2" t="n">
+        <v>-60.06</v>
       </c>
       <c r="W36" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO/COMERCIAL</t>
-        </is>
-      </c>
-      <c r="X36" t="inlineStr">
-        <is>
-          <t>15/05/2026</t>
-        </is>
+          <t>FROTA TERCEIRO PRUDENTE</t>
+        </is>
+      </c>
+      <c r="X36" s="3" t="n">
+        <v>46157</v>
       </c>
       <c r="Y36" t="inlineStr"/>
       <c r="Z36" t="inlineStr"/>
@@ -5533,32 +5470,32 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
@@ -5586,24 +5523,22 @@
           <t>TRPED290426</t>
         </is>
       </c>
-      <c r="T37" t="n">
+      <c r="T37" s="2" t="n">
         <v>42.61</v>
       </c>
-      <c r="U37" t="n">
-        <v>42.61</v>
-      </c>
-      <c r="V37" t="n">
-        <v>42.61</v>
+      <c r="U37" s="2" t="n">
+        <v>-42.61</v>
+      </c>
+      <c r="V37" s="2" t="n">
+        <v>-42.61</v>
       </c>
       <c r="W37" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO/COMERCIAL</t>
-        </is>
-      </c>
-      <c r="X37" t="inlineStr">
-        <is>
-          <t>15/05/2026</t>
-        </is>
+          <t>FROTA TERCEIRO PRUDENTE</t>
+        </is>
+      </c>
+      <c r="X37" s="3" t="n">
+        <v>46157</v>
       </c>
       <c r="Y37" t="inlineStr"/>
       <c r="Z37" t="inlineStr"/>
@@ -5673,32 +5608,32 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
@@ -5726,24 +5661,22 @@
           <t>TRPED300426</t>
         </is>
       </c>
-      <c r="T38" t="n">
+      <c r="T38" s="2" t="n">
         <v>97.51000000000001</v>
       </c>
-      <c r="U38" t="n">
-        <v>97.51000000000001</v>
-      </c>
-      <c r="V38" t="n">
-        <v>97.51000000000001</v>
+      <c r="U38" s="2" t="n">
+        <v>-97.51000000000001</v>
+      </c>
+      <c r="V38" s="2" t="n">
+        <v>-97.51000000000001</v>
       </c>
       <c r="W38" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO/COMERCIAL</t>
-        </is>
-      </c>
-      <c r="X38" t="inlineStr">
-        <is>
-          <t>15/05/2026</t>
-        </is>
+          <t>FROTA TERCEIRO PRUDENTE</t>
+        </is>
+      </c>
+      <c r="X38" s="3" t="n">
+        <v>46157</v>
       </c>
       <c r="Y38" t="inlineStr"/>
       <c r="Z38" t="inlineStr"/>
@@ -5866,24 +5799,22 @@
           <t>00492369</t>
         </is>
       </c>
-      <c r="T39" t="n">
+      <c r="T39" s="2" t="n">
         <v>471.95</v>
       </c>
-      <c r="U39" t="n">
-        <v>471.95</v>
-      </c>
-      <c r="V39" t="n">
-        <v>471.95</v>
+      <c r="U39" s="2" t="n">
+        <v>-471.95</v>
+      </c>
+      <c r="V39" s="2" t="n">
+        <v>-471.95</v>
       </c>
       <c r="W39" t="inlineStr">
         <is>
           <t>ADMINISTRATIVO/COMERCIAL</t>
         </is>
       </c>
-      <c r="X39" t="inlineStr">
-        <is>
-          <t>19/05/2026</t>
-        </is>
+      <c r="X39" s="3" t="n">
+        <v>46161</v>
       </c>
       <c r="Y39" t="inlineStr"/>
       <c r="Z39" t="inlineStr"/>
@@ -6006,24 +5937,22 @@
           <t>56531</t>
         </is>
       </c>
-      <c r="T40" t="n">
+      <c r="T40" s="2" t="n">
         <v>2275.49</v>
       </c>
-      <c r="U40" t="n">
-        <v>2275.49</v>
-      </c>
-      <c r="V40" t="n">
-        <v>2275.49</v>
+      <c r="U40" s="2" t="n">
+        <v>-2275.49</v>
+      </c>
+      <c r="V40" s="2" t="n">
+        <v>-2275.49</v>
       </c>
       <c r="W40" t="inlineStr">
         <is>
           <t>ADMINISTRATIVO/COMERCIAL</t>
         </is>
       </c>
-      <c r="X40" t="inlineStr">
-        <is>
-          <t>19/05/2026</t>
-        </is>
+      <c r="X40" s="3" t="n">
+        <v>46161</v>
       </c>
       <c r="Y40" t="inlineStr"/>
       <c r="Z40" t="inlineStr"/>
@@ -6146,24 +6075,22 @@
           <t>RETFED042026GSL01</t>
         </is>
       </c>
-      <c r="T41" t="n">
+      <c r="T41" s="2" t="n">
         <v>338.81</v>
       </c>
-      <c r="U41" t="n">
-        <v>338.81</v>
-      </c>
-      <c r="V41" t="n">
-        <v>338.81</v>
+      <c r="U41" s="2" t="n">
+        <v>-338.81</v>
+      </c>
+      <c r="V41" s="2" t="n">
+        <v>-338.81</v>
       </c>
       <c r="W41" t="inlineStr">
         <is>
           <t>ADMINISTRATIVO/COMERCIAL</t>
         </is>
       </c>
-      <c r="X41" t="inlineStr">
-        <is>
-          <t>19/05/2026</t>
-        </is>
+      <c r="X41" s="3" t="n">
+        <v>46161</v>
       </c>
       <c r="Y41" t="inlineStr"/>
       <c r="Z41" t="inlineStr"/>
@@ -6286,24 +6213,22 @@
           <t>TF15052026</t>
         </is>
       </c>
-      <c r="T42" t="n">
+      <c r="T42" s="2" t="n">
         <v>117.85</v>
       </c>
-      <c r="U42" t="n">
-        <v>117.85</v>
-      </c>
-      <c r="V42" t="n">
-        <v>117.85</v>
+      <c r="U42" s="2" t="n">
+        <v>-117.85</v>
+      </c>
+      <c r="V42" s="2" t="n">
+        <v>-117.85</v>
       </c>
       <c r="W42" t="inlineStr">
         <is>
           <t>ADMINISTRATIVO/COMERCIAL</t>
         </is>
       </c>
-      <c r="X42" t="inlineStr">
-        <is>
-          <t>20/05/2026</t>
-        </is>
+      <c r="X42" s="3" t="n">
+        <v>46162</v>
       </c>
       <c r="Y42" t="inlineStr"/>
       <c r="Z42" t="inlineStr"/>
@@ -6426,24 +6351,22 @@
           <t>4052878</t>
         </is>
       </c>
-      <c r="T43" t="n">
+      <c r="T43" s="2" t="n">
         <v>78.98999999999999</v>
       </c>
-      <c r="U43" t="n">
-        <v>78.98999999999999</v>
-      </c>
-      <c r="V43" t="n">
-        <v>78.98999999999999</v>
+      <c r="U43" s="2" t="n">
+        <v>-78.98999999999999</v>
+      </c>
+      <c r="V43" s="2" t="n">
+        <v>-78.98999999999999</v>
       </c>
       <c r="W43" t="inlineStr">
         <is>
           <t>ADMINISTRATIVO/COMERCIAL</t>
         </is>
       </c>
-      <c r="X43" t="inlineStr">
-        <is>
-          <t>21/05/2026</t>
-        </is>
+      <c r="X43" s="3" t="n">
+        <v>46163</v>
       </c>
       <c r="Y43" t="inlineStr"/>
       <c r="Z43" t="inlineStr"/>
@@ -6566,24 +6489,22 @@
           <t>PISCOFINS042026GSL</t>
         </is>
       </c>
-      <c r="T44" t="n">
+      <c r="T44" s="2" t="n">
         <v>40866.98</v>
       </c>
-      <c r="U44" t="n">
-        <v>40866.98</v>
-      </c>
-      <c r="V44" t="n">
-        <v>40866.98</v>
+      <c r="U44" s="2" t="n">
+        <v>-40866.98</v>
+      </c>
+      <c r="V44" s="2" t="n">
+        <v>-40866.98</v>
       </c>
       <c r="W44" t="inlineStr">
         <is>
           <t>ADMINISTRATIVO/COMERCIAL</t>
         </is>
       </c>
-      <c r="X44" t="inlineStr">
-        <is>
-          <t>22/05/2026</t>
-        </is>
+      <c r="X44" s="3" t="n">
+        <v>46164</v>
       </c>
       <c r="Y44" t="inlineStr"/>
       <c r="Z44" t="inlineStr"/>
@@ -6653,32 +6574,32 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
@@ -6706,24 +6627,22 @@
           <t>38381</t>
         </is>
       </c>
-      <c r="T45" t="n">
+      <c r="T45" s="2" t="n">
         <v>459.27</v>
       </c>
-      <c r="U45" t="n">
-        <v>459.27</v>
-      </c>
-      <c r="V45" t="n">
-        <v>459.27</v>
+      <c r="U45" s="2" t="n">
+        <v>-459.27</v>
+      </c>
+      <c r="V45" s="2" t="n">
+        <v>-459.27</v>
       </c>
       <c r="W45" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO/COMERCIAL</t>
-        </is>
-      </c>
-      <c r="X45" t="inlineStr">
-        <is>
-          <t>22/05/2026</t>
-        </is>
+          <t>FROTA TERCEIRO PRUDENTE</t>
+        </is>
+      </c>
+      <c r="X45" s="3" t="n">
+        <v>46164</v>
       </c>
       <c r="Y45" t="inlineStr"/>
       <c r="Z45" t="inlineStr"/>
@@ -6793,32 +6712,32 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="O46" t="inlineStr">
@@ -6846,24 +6765,22 @@
           <t>39075</t>
         </is>
       </c>
-      <c r="T46" t="n">
+      <c r="T46" s="2" t="n">
         <v>411.92</v>
       </c>
-      <c r="U46" t="n">
-        <v>411.92</v>
-      </c>
-      <c r="V46" t="n">
-        <v>411.92</v>
+      <c r="U46" s="2" t="n">
+        <v>-411.92</v>
+      </c>
+      <c r="V46" s="2" t="n">
+        <v>-411.92</v>
       </c>
       <c r="W46" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO/COMERCIAL</t>
-        </is>
-      </c>
-      <c r="X46" t="inlineStr">
-        <is>
-          <t>22/05/2026</t>
-        </is>
+          <t>FROTA TERCEIRO PRUDENTE</t>
+        </is>
+      </c>
+      <c r="X46" s="3" t="n">
+        <v>46164</v>
       </c>
       <c r="Y46" t="inlineStr"/>
       <c r="Z46" t="inlineStr"/>
@@ -6933,32 +6850,32 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="O47" t="inlineStr">
@@ -6986,24 +6903,22 @@
           <t>39669</t>
         </is>
       </c>
-      <c r="T47" t="n">
+      <c r="T47" s="2" t="n">
         <v>375.8</v>
       </c>
-      <c r="U47" t="n">
-        <v>375.8</v>
-      </c>
-      <c r="V47" t="n">
-        <v>375.8</v>
+      <c r="U47" s="2" t="n">
+        <v>-375.8</v>
+      </c>
+      <c r="V47" s="2" t="n">
+        <v>-375.8</v>
       </c>
       <c r="W47" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO/COMERCIAL</t>
-        </is>
-      </c>
-      <c r="X47" t="inlineStr">
-        <is>
-          <t>22/05/2026</t>
-        </is>
+          <t>FROTA TERCEIRO PRUDENTE</t>
+        </is>
+      </c>
+      <c r="X47" s="3" t="n">
+        <v>46164</v>
       </c>
       <c r="Y47" t="inlineStr"/>
       <c r="Z47" t="inlineStr"/>
@@ -7073,32 +6988,32 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="O48" t="inlineStr">
@@ -7126,24 +7041,22 @@
           <t>40269</t>
         </is>
       </c>
-      <c r="T48" t="n">
+      <c r="T48" s="2" t="n">
         <v>622.17</v>
       </c>
-      <c r="U48" t="n">
-        <v>622.17</v>
-      </c>
-      <c r="V48" t="n">
-        <v>622.17</v>
+      <c r="U48" s="2" t="n">
+        <v>-622.17</v>
+      </c>
+      <c r="V48" s="2" t="n">
+        <v>-622.17</v>
       </c>
       <c r="W48" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO/COMERCIAL</t>
-        </is>
-      </c>
-      <c r="X48" t="inlineStr">
-        <is>
-          <t>22/05/2026</t>
-        </is>
+          <t>FROTA TERCEIRO PRUDENTE</t>
+        </is>
+      </c>
+      <c r="X48" s="3" t="n">
+        <v>46164</v>
       </c>
       <c r="Y48" t="inlineStr"/>
       <c r="Z48" t="inlineStr"/>
@@ -7213,32 +7126,32 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
@@ -7266,24 +7179,22 @@
           <t>40887</t>
         </is>
       </c>
-      <c r="T49" t="n">
+      <c r="T49" s="2" t="n">
         <v>344.71</v>
       </c>
-      <c r="U49" t="n">
-        <v>344.71</v>
-      </c>
-      <c r="V49" t="n">
-        <v>344.71</v>
+      <c r="U49" s="2" t="n">
+        <v>-344.71</v>
+      </c>
+      <c r="V49" s="2" t="n">
+        <v>-344.71</v>
       </c>
       <c r="W49" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO/COMERCIAL</t>
-        </is>
-      </c>
-      <c r="X49" t="inlineStr">
-        <is>
-          <t>22/05/2026</t>
-        </is>
+          <t>FROTA TERCEIRO PRUDENTE</t>
+        </is>
+      </c>
+      <c r="X49" s="3" t="n">
+        <v>46164</v>
       </c>
       <c r="Y49" t="inlineStr"/>
       <c r="Z49" t="inlineStr"/>
@@ -7353,32 +7264,32 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
@@ -7406,24 +7317,22 @@
           <t>42494</t>
         </is>
       </c>
-      <c r="T50" t="n">
+      <c r="T50" s="2" t="n">
         <v>661.1900000000001</v>
       </c>
-      <c r="U50" t="n">
-        <v>661.1900000000001</v>
-      </c>
-      <c r="V50" t="n">
-        <v>661.1900000000001</v>
+      <c r="U50" s="2" t="n">
+        <v>-661.1900000000001</v>
+      </c>
+      <c r="V50" s="2" t="n">
+        <v>-661.1900000000001</v>
       </c>
       <c r="W50" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO/COMERCIAL</t>
-        </is>
-      </c>
-      <c r="X50" t="inlineStr">
-        <is>
-          <t>22/05/2026</t>
-        </is>
+          <t>FROTA TERCEIRO PRUDENTE</t>
+        </is>
+      </c>
+      <c r="X50" s="3" t="n">
+        <v>46164</v>
       </c>
       <c r="Y50" t="inlineStr"/>
       <c r="Z50" t="inlineStr"/>
@@ -7493,32 +7402,32 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="O51" t="inlineStr">
@@ -7546,24 +7455,22 @@
           <t>43245</t>
         </is>
       </c>
-      <c r="T51" t="n">
+      <c r="T51" s="2" t="n">
         <v>425.04</v>
       </c>
-      <c r="U51" t="n">
-        <v>425.04</v>
-      </c>
-      <c r="V51" t="n">
-        <v>425.04</v>
+      <c r="U51" s="2" t="n">
+        <v>-425.04</v>
+      </c>
+      <c r="V51" s="2" t="n">
+        <v>-425.04</v>
       </c>
       <c r="W51" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO/COMERCIAL</t>
-        </is>
-      </c>
-      <c r="X51" t="inlineStr">
-        <is>
-          <t>22/05/2026</t>
-        </is>
+          <t>FROTA TERCEIRO PRUDENTE</t>
+        </is>
+      </c>
+      <c r="X51" s="3" t="n">
+        <v>46164</v>
       </c>
       <c r="Y51" t="inlineStr"/>
       <c r="Z51" t="inlineStr"/>
@@ -7633,32 +7540,32 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="O52" t="inlineStr">
@@ -7686,24 +7593,22 @@
           <t>43802</t>
         </is>
       </c>
-      <c r="T52" t="n">
+      <c r="T52" s="2" t="n">
         <v>718.05</v>
       </c>
-      <c r="U52" t="n">
-        <v>718.05</v>
-      </c>
-      <c r="V52" t="n">
-        <v>718.05</v>
+      <c r="U52" s="2" t="n">
+        <v>-718.05</v>
+      </c>
+      <c r="V52" s="2" t="n">
+        <v>-718.05</v>
       </c>
       <c r="W52" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO/COMERCIAL</t>
-        </is>
-      </c>
-      <c r="X52" t="inlineStr">
-        <is>
-          <t>22/05/2026</t>
-        </is>
+          <t>FROTA TERCEIRO PRUDENTE</t>
+        </is>
+      </c>
+      <c r="X52" s="3" t="n">
+        <v>46164</v>
       </c>
       <c r="Y52" t="inlineStr"/>
       <c r="Z52" t="inlineStr"/>
@@ -7773,32 +7678,32 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="O53" t="inlineStr">
@@ -7826,24 +7731,22 @@
           <t>44340</t>
         </is>
       </c>
-      <c r="T53" t="n">
+      <c r="T53" s="2" t="n">
         <v>581.03</v>
       </c>
-      <c r="U53" t="n">
-        <v>581.03</v>
-      </c>
-      <c r="V53" t="n">
-        <v>581.03</v>
+      <c r="U53" s="2" t="n">
+        <v>-581.03</v>
+      </c>
+      <c r="V53" s="2" t="n">
+        <v>-581.03</v>
       </c>
       <c r="W53" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO/COMERCIAL</t>
-        </is>
-      </c>
-      <c r="X53" t="inlineStr">
-        <is>
-          <t>29/05/2026</t>
-        </is>
+          <t>FROTA TERCEIRO PRUDENTE</t>
+        </is>
+      </c>
+      <c r="X53" s="3" t="n">
+        <v>46171</v>
       </c>
       <c r="Y53" t="inlineStr"/>
       <c r="Z53" t="inlineStr"/>
@@ -7913,32 +7816,32 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="O54" t="inlineStr">
@@ -7966,24 +7869,22 @@
           <t>44941</t>
         </is>
       </c>
-      <c r="T54" t="n">
+      <c r="T54" s="2" t="n">
         <v>819.16</v>
       </c>
-      <c r="U54" t="n">
-        <v>819.16</v>
-      </c>
-      <c r="V54" t="n">
-        <v>819.16</v>
+      <c r="U54" s="2" t="n">
+        <v>-819.16</v>
+      </c>
+      <c r="V54" s="2" t="n">
+        <v>-819.16</v>
       </c>
       <c r="W54" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO/COMERCIAL</t>
-        </is>
-      </c>
-      <c r="X54" t="inlineStr">
-        <is>
-          <t>29/05/2026</t>
-        </is>
+          <t>FROTA TERCEIRO PRUDENTE</t>
+        </is>
+      </c>
+      <c r="X54" s="3" t="n">
+        <v>46171</v>
       </c>
       <c r="Y54" t="inlineStr"/>
       <c r="Z54" t="inlineStr"/>
@@ -8053,32 +7954,32 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>1.4.1.2</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>1.4.1.2 ADMINISTRATIVO</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="O55" t="inlineStr">
@@ -8106,24 +8007,22 @@
           <t>46451</t>
         </is>
       </c>
-      <c r="T55" t="n">
+      <c r="T55" s="2" t="n">
         <v>346.66</v>
       </c>
-      <c r="U55" t="n">
-        <v>346.66</v>
-      </c>
-      <c r="V55" t="n">
-        <v>346.66</v>
+      <c r="U55" s="2" t="n">
+        <v>-346.66</v>
+      </c>
+      <c r="V55" s="2" t="n">
+        <v>-346.66</v>
       </c>
       <c r="W55" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVO/COMERCIAL</t>
-        </is>
-      </c>
-      <c r="X55" t="inlineStr">
-        <is>
-          <t>29/05/2026</t>
-        </is>
+          <t>FROTA TERCEIRO PRUDENTE</t>
+        </is>
+      </c>
+      <c r="X55" s="3" t="n">
+        <v>46171</v>
       </c>
       <c r="Y55" t="inlineStr"/>
       <c r="Z55" t="inlineStr"/>

</xml_diff>